<commit_message>
feat(fhe_rl): integrate calibrated peak RAM model v3, vector packing, and clean repo
- Add compiler-faithful SIMD vector packing engine (packing.py, 100% ground-truth match)
- Integrate empirical calibration v3 (Log-Log for N<=16384, Proportional Ratio for N>16384)
- Plumb peak RAM constraint into MORL training and evaluation (NATO-SC and Lagrangian PID)
- Make runner and analysis scripts machine-portable using dynamic relative paths
- Add cross-validation and empirical audit tools (cv_strict.py, check_packing.py, rot_probe.py)
- Expand technical documentation (PEAK_RAM_INTEGRATION_AND_BUDGET_ANALYSIS.md)
- Purge obsolete one-time patch scripts, backup files, and terminal logs
</commit_message>
<xml_diff>
--- a/RL/job_logs.xlsx
+++ b/RL/job_logs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1015,6 +1015,120 @@
       <c r="O10" t="inlineStr">
         <is>
           <t>Algo: ppo | Method: lagrangian_od_ov | budget_encoding=raw | denom_factor=4 | num_envs=1 | budgets=None</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:47:53</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J11" t="n">
+        <v>21860</v>
+      </c>
+      <c r="K11" t="n">
+        <v>85</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>model_jobid_lagrangian_od_ov</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_lagrangian_od_ov</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: lagrangian_od_ov | budget_encoding=raw | denom_factor=4 | num_envs=2 | budgets=[1500, 2000, 2600, 1000000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>jobid</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:19:10</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2048</v>
+      </c>
+      <c r="E12" t="n">
+        <v>256</v>
+      </c>
+      <c r="F12" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J12" t="n">
+        <v>21860</v>
+      </c>
+      <c r="K12" t="n">
+        <v>85</v>
+      </c>
+      <c r="L12" t="n">
+        <v>50</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>model_jobid_lagrangian_od_ov</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>./tensorboard/model_jobid_lagrangian_od_ov</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Algo: ppo | Method: lagrangian_od_ov | budget_encoding=raw | denom_factor=4 | num_envs=2 | budgets=[1500, 2000, 2600, 1000000]</t>
         </is>
       </c>
     </row>

</xml_diff>